<commit_message>
Finish Java 27 article
</commit_message>
<xml_diff>
--- a/_drafts/jep-overview.xlsx
+++ b/_drafts/jep-overview.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hanno/Code/websites/hanno.codes/_drafts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33736F07-44D8-7D4F-A632-971275E48040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61AFCC03-9897-544E-BD56-7F3D26E9A82E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{D428FD44-A7BE-744F-BBBE-F876344939DC}"/>
+    <workbookView xWindow="8320" yWindow="3860" windowWidth="34560" windowHeight="21680" xr2:uid="{D428FD44-A7BE-744F-BBBE-F876344939DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -709,11 +709,11 @@
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="4.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31" customWidth="1"/>
-    <col min="4" max="4" width="21" style="2" customWidth="1"/>
+    <col min="3" max="3" width="32.5" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" style="2" customWidth="1"/>
     <col min="5" max="5" width="11.6640625" style="2" customWidth="1"/>
     <col min="6" max="6" width="12.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.5" style="2" customWidth="1"/>
+    <col min="7" max="7" width="11" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>